<commit_message>
Add US unit conversion rules for amz images
</commit_message>
<xml_diff>
--- a/skills/amz-create-image/templates/amz-create-image_workbook.xlsx
+++ b/skills/amz-create-image/templates/amz-create-image_workbook.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_说明" sheetId="1" r:id="Raf3cfc3536bf4930"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_阶段门禁" sheetId="2" r:id="R3369ba097814499a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_资料清单" sheetId="3" r:id="R5fc2650dffb244d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_竞品地图" sheetId="4" r:id="R4538fe5a43ea4be1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_关键词意图" sheetId="5" r:id="R9a06e29b572d43ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_评论痛点" sheetId="6" r:id="R63daa33f5c494b11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_主图需求" sheetId="7" r:id="Re5fcfd8521d349ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_副图需求" sheetId="8" r:id="R05da91dd27c642bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_主图副图参考图" sheetId="9" r:id="R1f3e35bf362a4111"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_主图副图验收" sheetId="10" r:id="Rec5d1743cd244d44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_A+参考图" sheetId="11" r:id="Rf2e797db75e3427b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_A+需求" sheetId="12" r:id="Ra79eefe37c6f4cab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_文案断行规则" sheetId="13" r:id="Rcbd64e02af5b42cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_版式尺寸规则" sheetId="14" r:id="Rbced27ed64c04a73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_合规检查" sheetId="15" r:id="Rc7b78e74cca9408e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_交付检查" sheetId="16" r:id="Re4dc556b0937429f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_说明" sheetId="1" r:id="Rfb882d2ff1024e8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_阶段门禁" sheetId="2" r:id="R2ad6dc26ca2a43d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_资料清单" sheetId="3" r:id="Re01d0f4042784e93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_竞品地图" sheetId="4" r:id="R7ae12e0a203f4234"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_关键词意图" sheetId="5" r:id="R9c24163ca95841a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_评论痛点" sheetId="6" r:id="R32b801280ef14146"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_主图需求" sheetId="7" r:id="Rf1d05b9247ed4345"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_副图需求" sheetId="8" r:id="R4fa1776d27ea4298"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_主图副图参考图" sheetId="9" r:id="Rcc4f5c88e70847df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_主图副图验收" sheetId="10" r:id="R91510c4bed61431d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_A+参考图" sheetId="11" r:id="R0f3ccf1fa5244e0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_A+需求" sheetId="12" r:id="R49cadb4c05ce412d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_文案断行规则" sheetId="13" r:id="R876a1eb4939b40cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_版式尺寸规则" sheetId="14" r:id="Rbfc758a490494073"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_合规检查" sheetId="15" r:id="Ra01bf31f1abf461d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_交付检查" sheetId="16" r:id="Rcb39b12d19864a59"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -91,7 +91,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -148,6 +148,16 @@
         <x:fgColor rgb="FF1F2937"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F2937"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -170,7 +180,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="65">
+  <x:cellXfs count="72">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
@@ -315,6 +325,19 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1171,6 +1194,7 @@
     <x:col min="15" max="15" width="28" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="42" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="30" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
@@ -1286,6 +1310,9 @@
       <x:c r="Q4" s="61" t="str">
         <x:v>验收标准</x:v>
       </x:c>
+      <x:c r="R4" s="70" t="str">
+        <x:v>单位换算/美制输出</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="92" customHeight="1">
       <x:c r="A5" s="62" t="str">
@@ -1341,6 +1368,9 @@
       <x:c r="Q5" s="64" t="str">
         <x:v>手机端可读，品牌感统一</x:v>
       </x:c>
+      <x:c r="R5" s="67" t="str">
+        <x:v>A+参数若来自cm/kg，输出in/lb；cm × 0.3937 = in，kg × 2.20462 = lb</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="92" customHeight="1">
       <x:c r="A6" s="63" t="str">
@@ -1396,6 +1426,9 @@
       <x:c r="Q6" s="64" t="str">
         <x:v>不得写No drilling若需螺丝</x:v>
       </x:c>
+      <x:c r="R6" s="67" t="str">
+        <x:v>安装/尺寸/重量参数需换算；主文案优先美制</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="92" customHeight="1">
       <x:c r="A7" s="62" t="str">
@@ -1451,6 +1484,9 @@
       <x:c r="Q7" s="64" t="str">
         <x:v>参数准确，可验证</x:v>
       </x:c>
+      <x:c r="R7" s="67" t="str">
+        <x:v>接口尺寸/产品尺寸如有cm需输出in</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="92" customHeight="1">
       <x:c r="A8" s="63" t="str">
@@ -1506,6 +1542,9 @@
       <x:c r="Q8" s="64" t="str">
         <x:v>功能逻辑正确</x:v>
       </x:c>
+      <x:c r="R8" s="67" t="str">
+        <x:v>功能参数若含重量需kg→lb</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="92" customHeight="1">
       <x:c r="A9" s="62" t="str">
@@ -1561,6 +1600,9 @@
       <x:c r="Q9" s="64" t="str">
         <x:v>定位为accent/ambient light</x:v>
       </x:c>
+      <x:c r="R9" s="67" t="str">
+        <x:v>场景模块通常不写硬参数；若写需换算</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="92" customHeight="1">
       <x:c r="A10" s="63" t="str">
@@ -1615,6 +1657,9 @@
       </x:c>
       <x:c r="Q10" s="64" t="str">
         <x:v>步骤清楚，无误导</x:v>
+      </x:c>
+      <x:c r="R10" s="67" t="str">
+        <x:v>安装步骤尺寸线必须用in，原始cm可备注</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="92" customHeight="1">
@@ -1672,6 +1717,12 @@
       <x:c r="Q11" s="64" t="str">
         <x:v>清单与实物一致</x:v>
       </x:c>
+      <x:c r="R11" s="67" t="str">
+        <x:v>包装重量如有kg需输出lb，配件尺寸cm需输出in</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="R12" s="67"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2189,13 +2240,30 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="64" customHeight="1">
-      <x:c r="A13" s="43"/>
-      <x:c r="B13" s="43"/>
-      <x:c r="C13" s="43"/>
-      <x:c r="D13" s="43"/>
-      <x:c r="E13" s="43"/>
-      <x:c r="F13" s="43"/>
-      <x:c r="G13" s="43"/>
+      <x:c r="A13" s="71" t="str">
+        <x:v>单位换算/美制输出</x:v>
+      </x:c>
+      <x:c r="B13" s="71" t="str">
+        <x:v>适用于所有尺寸/重量参数</x:v>
+      </x:c>
+      <x:c r="C13" s="71" t="str">
+        <x:v>若原始值为cm/kg，图片输出换算为in/lb</x:v>
+      </x:c>
+      <x:c r="D13" s="71" t="str">
+        <x:v>保留原始值核对</x:v>
+      </x:c>
+      <x:c r="E13" s="71" t="str">
+        <x:v>尺寸图/安装图/包装图/对比表必须执行</x:v>
+      </x:c>
+      <x:c r="F13" s="71" t="str">
+        <x:v>cm × 0.3937 = in；kg × 2.20462 = lb</x:v>
+      </x:c>
+      <x:c r="G13" s="71" t="str">
+        <x:v>美国站主展示优先英寸/磅，避免只写公制</x:v>
+      </x:c>
+      <x:c r="H13" s="67" t="str">
+        <x:v>美工执行列需写明换算后数值和单位</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2420,6 +2488,23 @@
       </x:c>
       <x:c r="E15" s="64"/>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="67" t="str">
+        <x:v>单位换算</x:v>
+      </x:c>
+      <x:c r="B16" s="67" t="str">
+        <x:v>尺寸/重量已从cm/kg换算为英寸/磅in/lb，并保留原始值核对</x:v>
+      </x:c>
+      <x:c r="C16" s="67" t="str">
+        <x:v>美国站图片直接写cm/kg，或换算错误</x:v>
+      </x:c>
+      <x:c r="D16" s="67" t="str">
+        <x:v>待检查</x:v>
+      </x:c>
+      <x:c r="E16" s="67" t="str">
+        <x:v>cm × 0.3937 = in；kg × 2.20462 = lb</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2608,6 +2693,20 @@
         <x:v>品牌_产品_主图副图_A+补充需求稿_vX.xlsx 或 Final 完整版</x:v>
       </x:c>
       <x:c r="D14" s="64" t="str">
+        <x:v>待检查</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="67" t="str">
+        <x:v>单位换算检查</x:v>
+      </x:c>
+      <x:c r="B15" s="67" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="C15" s="67" t="str">
+        <x:v>所有尺寸/重量参数已按cm→in、kg→lb换算；cm × 0.3937 = in，kg × 2.20462 = lb；换算依据写明且原始值可核对</x:v>
+      </x:c>
+      <x:c r="D15" s="67" t="str">
         <x:v>待检查</x:v>
       </x:c>
     </x:row>
@@ -3271,6 +3370,26 @@
         <x:is>
           <x:t xml:space="preserve">主图/副图验收前不得要求上传</x:t>
         </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="67" t="str">
+        <x:v>尺寸/重量单位换算</x:v>
+      </x:c>
+      <x:c r="B17" s="67" t="str">
+        <x:v>涉及尺寸/重量必填</x:v>
+      </x:c>
+      <x:c r="C17" s="67" t="str">
+        <x:v>美国站图片参数输出</x:v>
+      </x:c>
+      <x:c r="D17" s="67" t="str">
+        <x:v>输入可为cm/kg；输出需换算为in/lb；cm × 0.3937 = in，kg × 2.20462 = lb</x:v>
+      </x:c>
+      <x:c r="E17" s="67" t="str">
+        <x:v>待换算</x:v>
+      </x:c>
+      <x:c r="F17" s="67" t="str">
+        <x:v>保留原始cm/kg，图片主展示优先用英寸/磅</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4058,6 +4177,7 @@
     <x:col min="15" max="15" width="28" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="42" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="34" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
@@ -4173,6 +4293,9 @@
       <x:c r="Q4" s="61" t="str">
         <x:v>遮挡禁区/验收</x:v>
       </x:c>
+      <x:c r="R4" s="70" t="str">
+        <x:v>单位换算/美制输出</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="92" customHeight="1">
       <x:c r="A5" s="62" t="str">
@@ -4228,6 +4351,9 @@
       <x:c r="Q5" s="64" t="str">
         <x:v>文字不得压住灯体/光效；留80px安全边距</x:v>
       </x:c>
+      <x:c r="R5" s="67" t="str">
+        <x:v>涉及尺寸/重量时：保留原始cm/kg，输出in/lb；cm × 0.3937 = in，kg × 2.20462 = lb</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="92" customHeight="1">
       <x:c r="A6" s="63" t="str">
@@ -4282,6 +4408,9 @@
       </x:c>
       <x:c r="Q6" s="64" t="str">
         <x:v>充电口、线材清晰；不得遮挡接口</x:v>
+      </x:c>
+      <x:c r="R6" s="67" t="str">
+        <x:v>续航/电池容量不换算；如出现重量需kg→lb</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="92" customHeight="1">
@@ -4339,6 +4468,9 @@
       <x:c r="Q7" s="64" t="str">
         <x:v>按钮说明不可过小；手机端可读</x:v>
       </x:c>
+      <x:c r="R7" s="67" t="str">
+        <x:v>如遥控尺寸/重量出现，需cm/kg→in/lb</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="92" customHeight="1">
       <x:c r="A8" s="63" t="str">
@@ -4394,6 +4526,9 @@
       <x:c r="Q8" s="64" t="str">
         <x:v>卡片不能遮挡主灯；参数必须准确</x:v>
       </x:c>
+      <x:c r="R8" s="67" t="str">
+        <x:v>如灯体尺寸/重量出现，需cm/kg→in/lb</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="92" customHeight="1">
       <x:c r="A9" s="62" t="str">
@@ -4449,6 +4584,9 @@
       <x:c r="Q9" s="64" t="str">
         <x:v>不得出现产品不能支持的安装方式</x:v>
       </x:c>
+      <x:c r="R9" s="67" t="str">
+        <x:v>如旋转尺寸/灯体长度出现，需cm→in</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="92" customHeight="1">
       <x:c r="A10" s="63" t="str">
@@ -4504,6 +4642,9 @@
       <x:c r="Q10" s="64" t="str">
         <x:v>场景真实，不要AI感过强</x:v>
       </x:c>
+      <x:c r="R10" s="67" t="str">
+        <x:v>场景图一般不写硬参数；若写尺寸需cm→in</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="92" customHeight="1">
       <x:c r="A11" s="62" t="str">
@@ -4559,6 +4700,12 @@
       <x:c r="Q11" s="64" t="str">
         <x:v>所有尺寸须可验证；图中文字不能拥挤</x:v>
       </x:c>
+      <x:c r="R11" s="67" t="str">
+        <x:v>尺寸图必须输出英寸in；包装重量如有kg需输出lb</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="R12" s="67"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>